<commit_message>
UX optimize part 1
</commit_message>
<xml_diff>
--- a/CMS deploy plan(ok).xlsx
+++ b/CMS deploy plan(ok).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dangkn1\fe-kt-latest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{737FA61E-383A-4B43-855E-F7D61C254D4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{152971DF-A334-4F83-95F0-537301AA5136}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="327">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="321">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -804,44 +804,7 @@
     <t>UAT-TEA-06</t>
   </si>
   <si>
-    <t>Gắn giáo trình vào lớp</t>
-  </si>
-  <si>
-    <t>Gắn Giáo trình học vào Lớp học phụ trách (Class Curriculum)</t>
-  </si>
-  <si>
-    <t>1) Truy cập menu "Giao bài (Assignments)" -&gt; chọn tab "Giáo trình theo lớp"
-2) Chọn một Lớp học trong danh sách lớp mình phụ trách
-3) Nhấn nút "+ Gắn giáo trình vào lớp"
-4) Chọn Giáo trình học trong danh sách (hệ thống tự động lọc các giáo trình cùng môn học với lớp)
-5) Nhấn nút "Xác nhận gắn giáo trình"</t>
-  </si>
-  <si>
-    <t>Lớp: Lớp Tiếng Anh KATA 01, Giáo trình: Giáo trình Starter KATA Vol 1</t>
-  </si>
-  <si>
-    <t>1) Hệ thống hiển thị thông báo: "Đã gắn giáo trình vào lớp thành công!"
-2) Dòng giáo trình xuất hiện ngay trên bảng danh sách giáo trình của lớp học
-3) Tất cả học sinh trong lớp này sẽ nhìn thấy lộ trình học của giáo trình trong tài khoản của mình</t>
-  </si>
-  <si>
     <t>UAT-TEA-07</t>
-  </si>
-  <si>
-    <t>Gỡ Giáo trình học khỏi Lớp học khi không còn sử dụng</t>
-  </si>
-  <si>
-    <t>1) Tại tab "Giáo trình theo lớp", chọn lớp học đang có giáo trình đã gắn
-2) Tìm giáo trình cần gỡ, nhấn nút "Gỡ khỏi lớp" (biểu tượng Thùng rác / Hủy gắn)
-3) Hộp thoại xác nhận xuất hiện hỏi: "Bạn có chắc chắn muốn gỡ giáo trình này khỏi lớp học?"
-4) Nhấn "Xác nhận gỡ"</t>
-  </si>
-  <si>
-    <t>Lớp: Lớp Tiếng Anh KATA 01, Giáo trình cần gỡ</t>
-  </si>
-  <si>
-    <t>1) Hệ thống hiển thị thông báo: "Đã gỡ giáo trình khỏi lớp"
-2) Giáo trình được xóa khỏi bảng danh sách của lớp học ngay lập tức</t>
   </si>
   <si>
     <t>UAT-TEA-08</t>
@@ -977,9 +940,6 @@
   <si>
     <t>1) Cửa sổ tiến độ giáo trình hiển thị thanh phần trăm (Progress Bar) sinh động, trực quan
 2) Dễ dàng nhận diện học sinh nào đã hoàn thành 100% giáo trình và học sinh nào đang chậm tiến độ để nhắc nhở</t>
-  </si>
-  <si>
-    <t>UAT-TEA-14</t>
   </si>
   <si>
     <t>Bảng xếp hạng lớp</t>
@@ -1325,12 +1285,27 @@
 2) Màn hình ngay lập tức chuyển hướng an toàn về trang cá nhân của học sinh (/student/my-exams hoặc /student/profile)
 3) Tuyệt đối không để lộ dữ liệu quản trị, đảm bảo tính bảo mật và trải nghiệm người dùng</t>
   </si>
+  <si>
+    <t>Hủy giao giáo trình</t>
+  </si>
+  <si>
+    <t>Hủy giáo trình đã giao (Cancel Assignment) khi cần ngừng cho học sinh làm bài</t>
+  </si>
+  <si>
+    <t>1) Tại bảng danh sách giáo trình đã giao, tìm bài thi muốn hủy
+2) Nhấn nút "Hủy bài" (Cancel)
+3) Hộp thoại cảnh báo xuất hiện hỏi xác nhận thao tác hủy bài thi
+4) Nhấn "Xác nhận hủy"</t>
+  </si>
+  <si>
+    <t>Giáo trình đang ở trạng thái Hoạt động</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1362,6 +1337,12 @@
       <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1775,7 +1756,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -2723,10 +2704,10 @@
         <v>194</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>13</v>
@@ -2735,26 +2716,26 @@
         <v>167</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="I34" s="4"/>
       <c r="J34" s="3"/>
     </row>
-    <row r="35" spans="1:10" ht="80.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" ht="69" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D35" s="7" t="s">
         <v>13</v>
@@ -2763,26 +2744,26 @@
         <v>167</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="I35" s="7"/>
       <c r="J35" s="6"/>
     </row>
-    <row r="36" spans="1:10" ht="92" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" ht="69" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D36" s="4" t="s">
         <v>13</v>
@@ -2791,26 +2772,26 @@
         <v>167</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="I36" s="4"/>
       <c r="J36" s="3"/>
     </row>
     <row r="37" spans="1:10" ht="69" x14ac:dyDescent="0.35">
       <c r="A37" s="5" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="D37" s="7" t="s">
         <v>13</v>
@@ -2819,26 +2800,26 @@
         <v>167</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="I37" s="7"/>
       <c r="J37" s="6"/>
     </row>
     <row r="38" spans="1:10" ht="69" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>217</v>
+        <v>317</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>218</v>
+        <v>318</v>
       </c>
       <c r="D38" s="4" t="s">
         <v>13</v>
@@ -2847,522 +2828,495 @@
         <v>167</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>219</v>
+        <v>319</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>220</v>
+        <v>320</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="I38" s="4"/>
       <c r="J38" s="3"/>
     </row>
-    <row r="39" spans="1:10" ht="69" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" ht="92" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="F39" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="B39" s="6" t="s">
+      <c r="G39" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="C39" s="6" t="s">
+      <c r="H39" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="D39" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E39" s="5" t="s">
+      <c r="I39" s="4"/>
+      <c r="J39" s="3"/>
+    </row>
+    <row r="40" spans="1:10" ht="80.5" x14ac:dyDescent="0.35">
+      <c r="A40" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="D40" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E40" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="F39" s="6" t="s">
-        <v>225</v>
-      </c>
-      <c r="G39" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="H39" s="6" t="s">
+      <c r="F40" s="6" t="s">
         <v>227</v>
       </c>
-      <c r="I39" s="7"/>
-      <c r="J39" s="6"/>
-    </row>
-    <row r="40" spans="1:10" ht="92" x14ac:dyDescent="0.35">
-      <c r="A40" s="2" t="s">
+      <c r="G40" s="6" t="s">
         <v>228</v>
       </c>
-      <c r="B40" s="3" t="s">
+      <c r="H40" s="6" t="s">
         <v>229</v>
       </c>
-      <c r="C40" s="3" t="s">
-        <v>230</v>
-      </c>
-      <c r="D40" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="F40" s="3" t="s">
-        <v>231</v>
-      </c>
-      <c r="G40" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="H40" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="I40" s="4"/>
-      <c r="J40" s="3"/>
+      <c r="I40" s="7"/>
+      <c r="J40" s="6"/>
     </row>
     <row r="41" spans="1:10" ht="80.5" x14ac:dyDescent="0.35">
       <c r="A41" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="H41" s="3" t="s">
         <v>234</v>
       </c>
-      <c r="B41" s="6" t="s">
-        <v>229</v>
-      </c>
-      <c r="C41" s="6" t="s">
+      <c r="I41" s="4"/>
+      <c r="J41" s="3"/>
+    </row>
+    <row r="42" spans="1:10" ht="80.5" x14ac:dyDescent="0.35">
+      <c r="A42" s="5" t="s">
         <v>235</v>
       </c>
-      <c r="D41" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E41" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="F41" s="6" t="s">
+      <c r="B42" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C42" s="6" t="s">
         <v>236</v>
       </c>
-      <c r="G41" s="6" t="s">
+      <c r="D42" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E42" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="H41" s="6" t="s">
+      <c r="F42" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="I41" s="7"/>
-      <c r="J41" s="6"/>
-    </row>
-    <row r="42" spans="1:10" ht="80.5" x14ac:dyDescent="0.35">
-      <c r="A42" s="2" t="s">
+      <c r="G42" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="B42" s="3" t="s">
+      <c r="H42" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="C42" s="3" t="s">
+      <c r="I42" s="7"/>
+      <c r="J42" s="6"/>
+    </row>
+    <row r="43" spans="1:10" ht="69" x14ac:dyDescent="0.35">
+      <c r="A43" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="D42" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="F42" s="3" t="s">
+      <c r="B43" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="C43" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="G42" s="3" t="s">
+      <c r="D43" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="F43" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="H42" s="3" t="s">
+      <c r="G43" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="I42" s="4"/>
-      <c r="J42" s="3"/>
-    </row>
-    <row r="43" spans="1:10" ht="80.5" x14ac:dyDescent="0.35">
-      <c r="A43" s="5" t="s">
+      <c r="H43" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="B43" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C43" s="6" t="s">
+      <c r="I43" s="4"/>
+      <c r="J43" s="3"/>
+    </row>
+    <row r="44" spans="1:10" ht="115" x14ac:dyDescent="0.35">
+      <c r="A44" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="D43" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E43" s="5" t="s">
+      <c r="B44" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="C44" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="F43" s="6" t="s">
+      <c r="D44" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="F44" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="G43" s="6" t="s">
+      <c r="G44" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="H43" s="6" t="s">
+      <c r="H44" s="6" t="s">
         <v>250</v>
       </c>
-      <c r="I43" s="7"/>
-      <c r="J43" s="6"/>
-    </row>
-    <row r="44" spans="1:10" ht="69" x14ac:dyDescent="0.35">
-      <c r="A44" s="2" t="s">
+      <c r="I44" s="7"/>
+      <c r="J44" s="6"/>
+    </row>
+    <row r="45" spans="1:10" ht="103.5" x14ac:dyDescent="0.35">
+      <c r="A45" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="B44" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="C44" s="3" t="s">
+      <c r="B45" s="3" t="s">
         <v>252</v>
       </c>
-      <c r="D44" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="F44" s="3" t="s">
+      <c r="C45" s="3" t="s">
         <v>253</v>
       </c>
-      <c r="G44" s="3" t="s">
+      <c r="D45" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="F45" s="3" t="s">
         <v>254</v>
       </c>
-      <c r="H44" s="3" t="s">
+      <c r="G45" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="I44" s="4"/>
-      <c r="J44" s="3"/>
-    </row>
-    <row r="45" spans="1:10" ht="115" x14ac:dyDescent="0.35">
-      <c r="A45" s="5" t="s">
+      <c r="H45" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="B45" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="C45" s="6" t="s">
+      <c r="I45" s="4"/>
+      <c r="J45" s="3"/>
+    </row>
+    <row r="46" spans="1:10" ht="92" x14ac:dyDescent="0.35">
+      <c r="A46" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="D45" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E45" s="5" t="s">
-        <v>247</v>
-      </c>
-      <c r="F45" s="6" t="s">
+      <c r="B46" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="G45" s="6" t="s">
+      <c r="C46" s="6" t="s">
         <v>259</v>
       </c>
-      <c r="H45" s="6" t="s">
+      <c r="D46" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="F46" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="I45" s="7"/>
-      <c r="J45" s="6"/>
-    </row>
-    <row r="46" spans="1:10" ht="103.5" x14ac:dyDescent="0.35">
-      <c r="A46" s="2" t="s">
+      <c r="G46" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="B46" s="3" t="s">
+      <c r="H46" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="C46" s="3" t="s">
+      <c r="I46" s="7"/>
+      <c r="J46" s="6"/>
+    </row>
+    <row r="47" spans="1:10" ht="103.5" x14ac:dyDescent="0.35">
+      <c r="A47" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="D46" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="F46" s="3" t="s">
+      <c r="B47" s="3" t="s">
         <v>264</v>
       </c>
-      <c r="G46" s="3" t="s">
+      <c r="C47" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="H46" s="3" t="s">
+      <c r="D47" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="F47" s="3" t="s">
         <v>266</v>
       </c>
-      <c r="I46" s="4"/>
-      <c r="J46" s="3"/>
-    </row>
-    <row r="47" spans="1:10" ht="92" x14ac:dyDescent="0.35">
-      <c r="A47" s="5" t="s">
+      <c r="G47" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="B47" s="6" t="s">
+      <c r="H47" s="3" t="s">
         <v>268</v>
       </c>
-      <c r="C47" s="6" t="s">
+      <c r="I47" s="4"/>
+      <c r="J47" s="3"/>
+    </row>
+    <row r="48" spans="1:10" ht="69" x14ac:dyDescent="0.35">
+      <c r="A48" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="D47" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E47" s="5" t="s">
-        <v>247</v>
-      </c>
-      <c r="F47" s="6" t="s">
+      <c r="B48" s="6" t="s">
         <v>270</v>
       </c>
-      <c r="G47" s="6" t="s">
+      <c r="C48" s="6" t="s">
         <v>271</v>
       </c>
-      <c r="H47" s="6" t="s">
+      <c r="D48" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="F48" s="6" t="s">
         <v>272</v>
       </c>
-      <c r="I47" s="7"/>
-      <c r="J47" s="6"/>
-    </row>
-    <row r="48" spans="1:10" ht="103.5" x14ac:dyDescent="0.35">
-      <c r="A48" s="2" t="s">
+      <c r="G48" s="6" t="s">
         <v>273</v>
       </c>
-      <c r="B48" s="3" t="s">
+      <c r="H48" s="6" t="s">
         <v>274</v>
       </c>
-      <c r="C48" s="3" t="s">
+      <c r="I48" s="7"/>
+      <c r="J48" s="6"/>
+    </row>
+    <row r="49" spans="1:10" ht="92" x14ac:dyDescent="0.35">
+      <c r="A49" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="D48" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="F48" s="3" t="s">
+      <c r="B49" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="G48" s="3" t="s">
+      <c r="C49" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="H48" s="3" t="s">
+      <c r="D49" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="F49" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="I48" s="4"/>
-      <c r="J48" s="3"/>
-    </row>
-    <row r="49" spans="1:10" ht="69" x14ac:dyDescent="0.35">
-      <c r="A49" s="5" t="s">
+      <c r="G49" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="H49" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="C49" s="6" t="s">
+      <c r="I49" s="4"/>
+      <c r="J49" s="3"/>
+    </row>
+    <row r="50" spans="1:10" ht="103.5" x14ac:dyDescent="0.35">
+      <c r="A50" s="5" t="s">
         <v>281</v>
       </c>
-      <c r="D49" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E49" s="5" t="s">
-        <v>247</v>
-      </c>
-      <c r="F49" s="6" t="s">
+      <c r="B50" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="G49" s="6" t="s">
+      <c r="C50" s="6" t="s">
         <v>283</v>
       </c>
-      <c r="H49" s="6" t="s">
+      <c r="D50" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E50" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="F50" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="I49" s="7"/>
-      <c r="J49" s="6"/>
-    </row>
-    <row r="50" spans="1:10" ht="92" x14ac:dyDescent="0.35">
-      <c r="A50" s="2" t="s">
+      <c r="G50" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="B50" s="3" t="s">
+      <c r="H50" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="C50" s="3" t="s">
+      <c r="I50" s="7"/>
+      <c r="J50" s="6"/>
+    </row>
+    <row r="51" spans="1:10" ht="69" x14ac:dyDescent="0.35">
+      <c r="A51" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="D50" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="F50" s="3" t="s">
+      <c r="B51" s="3" t="s">
         <v>288</v>
       </c>
-      <c r="G50" s="3" t="s">
+      <c r="C51" s="3" t="s">
         <v>289</v>
       </c>
-      <c r="H50" s="3" t="s">
+      <c r="D51" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="F51" s="3" t="s">
         <v>290</v>
       </c>
-      <c r="I50" s="4"/>
-      <c r="J50" s="3"/>
-    </row>
-    <row r="51" spans="1:10" ht="103.5" x14ac:dyDescent="0.35">
-      <c r="A51" s="5" t="s">
+      <c r="G51" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="B51" s="6" t="s">
+      <c r="H51" s="3" t="s">
         <v>292</v>
       </c>
-      <c r="C51" s="6" t="s">
+      <c r="I51" s="4"/>
+      <c r="J51" s="3"/>
+    </row>
+    <row r="52" spans="1:10" ht="103.5" x14ac:dyDescent="0.35">
+      <c r="A52" s="5" t="s">
         <v>293</v>
       </c>
-      <c r="D51" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E51" s="5" t="s">
-        <v>247</v>
-      </c>
-      <c r="F51" s="6" t="s">
+      <c r="B52" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="G51" s="6" t="s">
+      <c r="C52" s="6" t="s">
         <v>295</v>
       </c>
-      <c r="H51" s="6" t="s">
+      <c r="D52" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E52" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="F52" s="6" t="s">
         <v>296</v>
       </c>
-      <c r="I51" s="7"/>
-      <c r="J51" s="6"/>
-    </row>
-    <row r="52" spans="1:10" ht="69" x14ac:dyDescent="0.35">
-      <c r="A52" s="2" t="s">
+      <c r="G52" s="6" t="s">
         <v>297</v>
       </c>
-      <c r="B52" s="3" t="s">
+      <c r="H52" s="6" t="s">
         <v>298</v>
       </c>
-      <c r="C52" s="3" t="s">
+      <c r="I52" s="7"/>
+      <c r="J52" s="6"/>
+    </row>
+    <row r="53" spans="1:10" ht="92" x14ac:dyDescent="0.35">
+      <c r="A53" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="D52" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="F52" s="3" t="s">
+      <c r="B53" s="3" t="s">
         <v>300</v>
       </c>
-      <c r="G52" s="3" t="s">
+      <c r="C53" s="3" t="s">
         <v>301</v>
       </c>
-      <c r="H52" s="3" t="s">
+      <c r="D53" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="F53" s="3" t="s">
         <v>302</v>
       </c>
-      <c r="I52" s="4"/>
-      <c r="J52" s="3"/>
-    </row>
-    <row r="53" spans="1:10" ht="103.5" x14ac:dyDescent="0.35">
-      <c r="A53" s="5" t="s">
+      <c r="G53" s="3" t="s">
         <v>303</v>
       </c>
-      <c r="B53" s="6" t="s">
+      <c r="H53" s="3" t="s">
         <v>304</v>
       </c>
-      <c r="C53" s="6" t="s">
+      <c r="I53" s="4"/>
+      <c r="J53" s="3"/>
+    </row>
+    <row r="54" spans="1:10" ht="138" x14ac:dyDescent="0.35">
+      <c r="A54" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="D53" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E53" s="5" t="s">
-        <v>247</v>
-      </c>
-      <c r="F53" s="6" t="s">
+      <c r="B54" s="6" t="s">
         <v>306</v>
       </c>
-      <c r="G53" s="6" t="s">
+      <c r="C54" s="6" t="s">
         <v>307</v>
       </c>
-      <c r="H53" s="6" t="s">
+      <c r="D54" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E54" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="F54" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="I53" s="7"/>
-      <c r="J53" s="6"/>
-    </row>
-    <row r="54" spans="1:10" ht="92" x14ac:dyDescent="0.35">
-      <c r="A54" s="2" t="s">
+      <c r="G54" s="6" t="s">
         <v>309</v>
       </c>
-      <c r="B54" s="3" t="s">
+      <c r="H54" s="6" t="s">
         <v>310</v>
       </c>
-      <c r="C54" s="3" t="s">
+      <c r="I54" s="7"/>
+      <c r="J54" s="6"/>
+    </row>
+    <row r="55" spans="1:10" ht="69" x14ac:dyDescent="0.35">
+      <c r="A55" s="2" t="s">
         <v>311</v>
       </c>
-      <c r="D54" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="F54" s="3" t="s">
+      <c r="B55" s="3" t="s">
         <v>312</v>
       </c>
-      <c r="G54" s="3" t="s">
+      <c r="C55" s="3" t="s">
         <v>313</v>
       </c>
-      <c r="H54" s="3" t="s">
+      <c r="D55" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="F55" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="I54" s="4"/>
-      <c r="J54" s="3"/>
-    </row>
-    <row r="55" spans="1:10" ht="138" x14ac:dyDescent="0.35">
-      <c r="A55" s="5" t="s">
+      <c r="G55" s="3" t="s">
         <v>315</v>
       </c>
-      <c r="B55" s="6" t="s">
+      <c r="H55" s="3" t="s">
         <v>316</v>
       </c>
-      <c r="C55" s="6" t="s">
-        <v>317</v>
-      </c>
-      <c r="D55" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E55" s="5" t="s">
-        <v>247</v>
-      </c>
-      <c r="F55" s="6" t="s">
-        <v>318</v>
-      </c>
-      <c r="G55" s="6" t="s">
-        <v>319</v>
-      </c>
-      <c r="H55" s="6" t="s">
-        <v>320</v>
-      </c>
-      <c r="I55" s="7"/>
-      <c r="J55" s="6"/>
-    </row>
-    <row r="56" spans="1:10" ht="69" x14ac:dyDescent="0.35">
-      <c r="A56" s="2" t="s">
-        <v>321</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>322</v>
-      </c>
-      <c r="C56" s="3" t="s">
-        <v>323</v>
-      </c>
-      <c r="D56" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E56" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="F56" s="3" t="s">
-        <v>324</v>
-      </c>
-      <c r="G56" s="3" t="s">
-        <v>325</v>
-      </c>
-      <c r="H56" s="3" t="s">
-        <v>326</v>
-      </c>
-      <c r="I56" s="4"/>
-      <c r="J56" s="3"/>
+      <c r="I55" s="4"/>
+      <c r="J55" s="3"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>